<commit_message>
Added final advanced analysis and visualizations
</commit_message>
<xml_diff>
--- a/WB_Election_Results_2026.xlsx
+++ b/WB_Election_Results_2026.xlsx
@@ -1796,822 +1796,825 @@
     <t>CHANDRANATH SINHA</t>
   </si>
   <si>
+    <t>BIDHAN CHANDRA MAJHI</t>
+  </si>
+  <si>
+    <t>DEBASIS OJHA (HAKU DA)</t>
+  </si>
+  <si>
+    <t>KRISHNA KANTA SAHA</t>
+  </si>
+  <si>
+    <t>DUDH KUMAR MONDAL</t>
+  </si>
+  <si>
+    <t>DHRUBA SAHA</t>
+  </si>
+  <si>
+    <t>FAYEZUL HAQUE (KAJAL SK)</t>
+  </si>
+  <si>
+    <t>RAJENDRA PRASAD SINGH(RAJU SINGH)</t>
+  </si>
+  <si>
+    <t>DR. MOSARRAF HOSSAIN</t>
+  </si>
+  <si>
+    <t>Bharatiya Janata Party</t>
+  </si>
+  <si>
+    <t>All India Trinamool Congress</t>
+  </si>
+  <si>
+    <t>Indian National Congress</t>
+  </si>
+  <si>
+    <t>Aam Janata Unnayan party</t>
+  </si>
+  <si>
+    <t>Communist Party of India (Marxist)</t>
+  </si>
+  <si>
+    <t>All India Secular Front</t>
+  </si>
+  <si>
+    <t>Won</t>
+  </si>
+  <si>
+    <t>Leading</t>
+  </si>
+  <si>
+    <t>ADHIKARY PARESH CHANDRA</t>
+  </si>
+  <si>
+    <t>DR. SABLU BARMAN</t>
+  </si>
+  <si>
+    <t>PARTHA PRATIM RAY</t>
+  </si>
+  <si>
+    <t>AVIJIT DE BHOWMIK</t>
+  </si>
+  <si>
+    <t>HARIHAR DAS</t>
+  </si>
+  <si>
+    <t>ASHUTOSH BARMA</t>
+  </si>
+  <si>
+    <t>UDAYAN GUHA</t>
+  </si>
+  <si>
+    <t>SAILENDRA NATH BARMA</t>
+  </si>
+  <si>
+    <t>SHIBSANKAR PAUL</t>
+  </si>
+  <si>
+    <t>RAJEEV TIRKEY</t>
+  </si>
+  <si>
+    <t>BIRENDRA BARA (ORAON)</t>
+  </si>
+  <si>
+    <t>SUMAN KANJILAL</t>
+  </si>
+  <si>
+    <t>SUBHASH CHANDRA ROY</t>
+  </si>
+  <si>
+    <t>JAYPRAKASH TOPPO</t>
+  </si>
+  <si>
+    <t>NIRMAL CHANDRA ROY</t>
+  </si>
+  <si>
+    <t>RAMMOHAN RAY</t>
+  </si>
+  <si>
+    <t>KRISHNA DAS</t>
+  </si>
+  <si>
+    <t>SWAPNA BARMAN</t>
+  </si>
+  <si>
+    <t>RANJAN SIL SHARMA</t>
+  </si>
+  <si>
+    <t>BULU CHIK BARAIK</t>
+  </si>
+  <si>
+    <t>SANJAY KUJUR</t>
+  </si>
+  <si>
+    <t>RUDEN SADA LEPCHA</t>
+  </si>
+  <si>
+    <t>BIJOY KUMAR RAI</t>
+  </si>
+  <si>
+    <t>AMAR LAMA</t>
+  </si>
+  <si>
+    <t>SHANKAR MALAKAR</t>
+  </si>
+  <si>
+    <t>GOUTAM DEB</t>
+  </si>
+  <si>
+    <t>REENA TOPNO EKKA</t>
+  </si>
+  <si>
+    <t>SANKAR ADHIKARI</t>
+  </si>
+  <si>
+    <t>CHITRAJIT ROY</t>
+  </si>
+  <si>
+    <t>SARAJIT BISWAS</t>
+  </si>
+  <si>
+    <t>MANOJ KUMAR JAIN</t>
+  </si>
+  <si>
+    <t>GOUTAM PAUL</t>
+  </si>
+  <si>
+    <t>SATYAJIT BARMAN</t>
+  </si>
+  <si>
+    <t>NITAI BAISHYA</t>
+  </si>
+  <si>
+    <t>KRISHNA KALYANI</t>
+  </si>
+  <si>
+    <t>SABITA BARMAN</t>
+  </si>
+  <si>
+    <t>REKHA ROY</t>
+  </si>
+  <si>
+    <t>SUBHENDU SARKAR</t>
+  </si>
+  <si>
+    <t>ARPITA GHOSH</t>
+  </si>
+  <si>
+    <t>CHINTAMANI BIHA</t>
+  </si>
+  <si>
+    <t>Goutam Das</t>
+  </si>
+  <si>
+    <t>DEBABRATA MAJUMDER</t>
+  </si>
+  <si>
+    <t>AMAL KISKU</t>
+  </si>
+  <si>
+    <t>PRASENJIT DAS</t>
+  </si>
+  <si>
+    <t>RATAN DAS</t>
+  </si>
+  <si>
+    <t>MAUSAM B NOOR</t>
+  </si>
+  <si>
+    <t>ABISHEK SINGHANIA</t>
+  </si>
+  <si>
+    <t>KABITA MANDAL</t>
+  </si>
+  <si>
+    <t>LIPIKA BARMAN GHOSH</t>
+  </si>
+  <si>
+    <t>ASIS KUNDU (PATA)</t>
+  </si>
+  <si>
+    <t>NIBARAN GHOSH</t>
+  </si>
+  <si>
+    <t>ABDUL HANNAN</t>
+  </si>
+  <si>
+    <t>CHANDANA SARKAR</t>
+  </si>
+  <si>
+    <t>SUNIL CHOWDHURI</t>
+  </si>
+  <si>
+    <t>MD NAJME ALAM</t>
+  </si>
+  <si>
+    <t>MAHABIR GHOSH</t>
+  </si>
+  <si>
+    <t>JAKIR HOSSAIN</t>
+  </si>
+  <si>
+    <t>NASIR SAIKH</t>
+  </si>
+  <si>
+    <t>TAPAS KUMAR CHAKRABORTY</t>
+  </si>
+  <si>
+    <t>TOUHIDUR RAHAMAN SUMAN</t>
+  </si>
+  <si>
+    <t>MAHAMUDAL HASAN</t>
+  </si>
+  <si>
+    <t>ABDUL SOUMIK HOSSAIN</t>
+  </si>
+  <si>
+    <t>SHAONI SINGHA ROY</t>
+  </si>
+  <si>
+    <t>PRONAB CHANDRA DAS</t>
+  </si>
+  <si>
+    <t>ASHIS MARJIT</t>
+  </si>
+  <si>
+    <t>PROTIMA RAJAK</t>
+  </si>
+  <si>
+    <t>APURBA SARKAR (DAVID)</t>
+  </si>
+  <si>
+    <t>ANAMIKA GHOSH</t>
+  </si>
+  <si>
+    <t>BAPAN GHOSH</t>
+  </si>
+  <si>
+    <t>RABIUL ALAM CHOWDHURY</t>
+  </si>
+  <si>
+    <t>ADHIR RANJAN CHOWDHURY</t>
+  </si>
+  <si>
+    <t>BIJOY SEKH</t>
+  </si>
+  <si>
+    <t>RANA MANDAL</t>
+  </si>
+  <si>
+    <t>IANUS ALI SARKAR</t>
+  </si>
+  <si>
+    <t>SOHAM CHAKRABORTY</t>
+  </si>
+  <si>
+    <t>DILIP KUMAR PODDAR</t>
+  </si>
+  <si>
+    <t>ANIMA DUTTA</t>
+  </si>
+  <si>
+    <t>KALLOL KHAN</t>
+  </si>
+  <si>
+    <t>SAIKAT SARKAR</t>
+  </si>
+  <si>
+    <t>SOMNATH DUTTA</t>
+  </si>
+  <si>
+    <t>PUNDARIKAKSHYA SAHA</t>
+  </si>
+  <si>
+    <t>UJJAL BISWAS</t>
+  </si>
+  <si>
+    <t>BRAJAKISHORE GOSWAMI</t>
+  </si>
+  <si>
+    <t>TAPAS KUMAR GHOSH</t>
+  </si>
+  <si>
+    <t>SAMIR KUMAR PODDAR</t>
+  </si>
+  <si>
+    <t>BARNALI DEY ROY</t>
+  </si>
+  <si>
+    <t>SOUGATA KUMAR BURMAN</t>
+  </si>
+  <si>
+    <t>SUBHANKAR SINGHA (JISHU)</t>
+  </si>
+  <si>
+    <t>DR. ATINDRA NATH MONDAL</t>
+  </si>
+  <si>
+    <t>DR. RAJIB BISWAS.</t>
+  </si>
+  <si>
+    <t>MADHUPARNA THAKUR</t>
+  </si>
+  <si>
+    <t>BISWAJIT DAS</t>
+  </si>
+  <si>
+    <t>RITUPARNA ADDHYA</t>
+  </si>
+  <si>
+    <t>NAROTTAM BISWAS</t>
+  </si>
+  <si>
+    <t>TARAK SAHA</t>
+  </si>
+  <si>
+    <t>SUKRITI KUMAR SARKAR</t>
+  </si>
+  <si>
+    <t>JYOTI PRIYA MALLICK</t>
+  </si>
+  <si>
+    <t>NARAYAN GOSWAMI</t>
+  </si>
+  <si>
+    <t>ARINDAM DEY</t>
+  </si>
+  <si>
+    <t>SUBODH ADHIKARY</t>
+  </si>
+  <si>
+    <t>SANAT DEY</t>
+  </si>
+  <si>
+    <t>AMIT GUPTA</t>
+  </si>
+  <si>
+    <t>SOMENATH SHYAM ICHINI</t>
+  </si>
+  <si>
+    <t>TRINANKUR BHATTACHARJEE</t>
+  </si>
+  <si>
+    <t>RAJ CHAKRABORTY (RAJU)</t>
+  </si>
+  <si>
+    <t>DEVADEEP PUROHIT</t>
+  </si>
+  <si>
+    <t>CHANDRIMA BHATTACHARYA</t>
+  </si>
+  <si>
+    <t>TIRTHANKAR GHOSH</t>
+  </si>
+  <si>
+    <t>ARUP CHOUDHURY (PULAK)</t>
+  </si>
+  <si>
+    <t>SAYANTIKA BANERJEE</t>
+  </si>
+  <si>
+    <t>BRATYABRATA BASU</t>
+  </si>
+  <si>
+    <t>PIYUSH KANODIA</t>
+  </si>
+  <si>
+    <t>SUJIT BOSE</t>
+  </si>
+  <si>
+    <t>ADITI MUNSHI</t>
+  </si>
+  <si>
+    <t>RATHIN GHOSH</t>
+  </si>
+  <si>
+    <t>SABYASACHI DUTTA</t>
+  </si>
+  <si>
+    <t>MD MOFIDUL HOQUE SAHAJI MINTU</t>
+  </si>
+  <si>
+    <t>PIYARUL ISLAM</t>
+  </si>
+  <si>
+    <t>RUDRENDRA PATRA</t>
+  </si>
+  <si>
+    <t>JHARNA SARDAR</t>
+  </si>
+  <si>
+    <t>DR. SOURYA BANERJEE</t>
+  </si>
+  <si>
+    <t>MD. MUSA KAREMULLA</t>
+  </si>
+  <si>
+    <t>ANANDA SARKAR</t>
+  </si>
+  <si>
+    <t>SUBRATA MONDAL</t>
+  </si>
+  <si>
+    <t>BIKASH SARDAR</t>
+  </si>
+  <si>
+    <t>MADHABI MAHALDER</t>
+  </si>
+  <si>
+    <t>ASIT KUMAR HALDAR</t>
+  </si>
+  <si>
+    <t>MANTURAM PAKHIRA</t>
+  </si>
+  <si>
+    <t>BANKIM CHANDRA HAZRA</t>
+  </si>
+  <si>
+    <t>ABANI NASKAR</t>
+  </si>
+  <si>
+    <t>PALASH RANA</t>
+  </si>
+  <si>
+    <t>MALLIKA PAIK W/O - ASHOK PAIK</t>
+  </si>
+  <si>
+    <t>ALOKE HALDER</t>
+  </si>
+  <si>
+    <t>TUMPA SARDAR</t>
+  </si>
+  <si>
+    <t>Prasanta Bayen</t>
+  </si>
+  <si>
+    <t>ARABUL ISLAM</t>
+  </si>
+  <si>
+    <t>BISWAJIT PAUL</t>
+  </si>
+  <si>
+    <t>UTTAM KUMAR BANIK</t>
+  </si>
+  <si>
+    <t>GOURSUNDAR GHOSH</t>
+  </si>
+  <si>
+    <t>DIPAK KUMAR HALDER</t>
+  </si>
+  <si>
+    <t>JAHANGIR KHAN</t>
+  </si>
+  <si>
+    <t>SOMASHREE BETAL</t>
+  </si>
+  <si>
+    <t>ABHIJIT SARDAR</t>
+  </si>
+  <si>
+    <t>ARUNDHUTI MAITRA(LOVELY)</t>
+  </si>
+  <si>
+    <t>SAOKAT MOLLA</t>
+  </si>
+  <si>
+    <t>BANERJEE SANDIP</t>
+  </si>
+  <si>
+    <t>DEBABRATA MAJUMDAR (MALAY)</t>
+  </si>
+  <si>
+    <t>FIRDOUSI BEGAM</t>
+  </si>
+  <si>
+    <t>AROOP BISWAS</t>
+  </si>
+  <si>
+    <t>SUBHASISH CHAKRABORTY</t>
+  </si>
+  <si>
+    <t>RATNA CHATTERJEE</t>
+  </si>
+  <si>
+    <t>TAMANATH BHOWMICK</t>
+  </si>
+  <si>
+    <t>DR TARUN KUMAR ADAK</t>
+  </si>
+  <si>
+    <t>BIR BAHADUR SINGH</t>
+  </si>
+  <si>
+    <t>RAKESH SINGH</t>
+  </si>
+  <si>
+    <t>MAMATA BANERJEE</t>
+  </si>
+  <si>
+    <t>DEBASISH KUMAR (DEBA)</t>
+  </si>
+  <si>
+    <t>SHATORUPA</t>
+  </si>
+  <si>
+    <t>SANTOSH KUMAR PATHAK</t>
+  </si>
+  <si>
+    <t>DR. PRIYANKA TIBREWAL</t>
+  </si>
+  <si>
+    <t>PARTHA CHAUDHURY</t>
+  </si>
+  <si>
+    <t>VIJAY UPADHYAY</t>
+  </si>
+  <si>
+    <t>SHASHI PANJA</t>
+  </si>
+  <si>
+    <t>SHRREYA PANDE</t>
+  </si>
+  <si>
+    <t>ATIN GHOSH</t>
+  </si>
+  <si>
+    <t>KAILASH KUMAR MISHRA</t>
+  </si>
+  <si>
+    <t>GAUTAM CHOWDHURY</t>
+  </si>
+  <si>
+    <t>BIPLAB KUMAR MANDAL</t>
+  </si>
+  <si>
+    <t>DR. RANA CHATTERJEE</t>
+  </si>
+  <si>
+    <t>SHYAMAL KUMAR HATI</t>
+  </si>
+  <si>
+    <t>BARNALI DHALI NASKAR</t>
+  </si>
+  <si>
+    <t>RANJAN PAUL</t>
+  </si>
+  <si>
+    <t>RUDRA PROSAD BANERJEE</t>
+  </si>
+  <si>
+    <t>BIMAL KUMAR DAS</t>
+  </si>
+  <si>
+    <t>SWAMI MANGALANANDA PURI</t>
+  </si>
+  <si>
+    <t>NADEBASI JANA</t>
+  </si>
+  <si>
+    <t>PRAMANSHU RANA</t>
+  </si>
+  <si>
+    <t>SUKANTA KUMAR PAUL</t>
+  </si>
+  <si>
+    <t>PROBHAKAR PANDIT</t>
+  </si>
+  <si>
+    <t>SUBIR CHATTERJEE (TINKAI)</t>
+  </si>
+  <si>
+    <t>GOBINDA HAZRA</t>
+  </si>
+  <si>
+    <t>SIRSANYA BANDOPADHYAY</t>
+  </si>
+  <si>
+    <t>TANMOY GHOSH</t>
+  </si>
+  <si>
+    <t>ARINDAM GUIN (BUBAI)</t>
+  </si>
+  <si>
+    <t>BECHARAM MANNA</t>
+  </si>
+  <si>
+    <t>Indranil Sen</t>
+  </si>
+  <si>
+    <t>DEBANGSHU BHATTACHARYA</t>
+  </si>
+  <si>
+    <t>RANJAN DHARA</t>
+  </si>
+  <si>
+    <t>SAMIR CHAKRABORTY</t>
+  </si>
+  <si>
+    <t>BIDESH RANJAN BOSE</t>
+  </si>
+  <si>
+    <t>DEBASISH MUKHERJEE</t>
+  </si>
+  <si>
+    <t>SNEHASIS CHAKRABORTY</t>
+  </si>
+  <si>
+    <t>KARABI MANNA</t>
+  </si>
+  <si>
+    <t>BARNALI DAS</t>
+  </si>
+  <si>
+    <t>RAMENDU SINHARAY</t>
+  </si>
+  <si>
+    <t>PARTHA HAZARI</t>
+  </si>
+  <si>
+    <t>BAG MITA</t>
+  </si>
+  <si>
+    <t>DR. NIRMAL MAJI</t>
+  </si>
+  <si>
+    <t>PALASH KUMAR ROY</t>
+  </si>
+  <si>
+    <t>DIPENDRA NARAYAN ROY</t>
+  </si>
+  <si>
+    <t>ASHIM KUMAR MAJI</t>
+  </si>
+  <si>
+    <t>SIRAJ KHAN</t>
+  </si>
+  <si>
+    <t>CHANDAN MONDAL</t>
+  </si>
+  <si>
+    <t>SUKUMAR DE</t>
+  </si>
+  <si>
+    <t>TILAK KUMAR CHAKRABORTY</t>
+  </si>
+  <si>
+    <t>TAPASI MONDAL</t>
+  </si>
+  <si>
+    <t>PABITRA KAR</t>
+  </si>
+  <si>
+    <t>UTTAM BARIK</t>
+  </si>
+  <si>
+    <t>PIJUS KANTI PANDA</t>
+  </si>
+  <si>
+    <t>DEBASIS BHUNYA</t>
+  </si>
+  <si>
+    <t>MANAB KUMAR PARUA</t>
+  </si>
+  <si>
+    <t>RABIN CHANDRA MANDAL</t>
+  </si>
+  <si>
+    <t>TARUN KUMAR JANA</t>
+  </si>
+  <si>
+    <t>AKHIL GIRI</t>
+  </si>
+  <si>
+    <t>TARUN KUMAR MAITY</t>
+  </si>
+  <si>
+    <t>MANIK MAITI</t>
+  </si>
+  <si>
+    <t>DULAL MURMU</t>
+  </si>
+  <si>
+    <t>AJIT MAHATA</t>
+  </si>
+  <si>
+    <t>MONGAL SAREN</t>
+  </si>
+  <si>
+    <t>RAMJIBAN MANDI</t>
+  </si>
+  <si>
+    <t>PRADIP SARKAR</t>
+  </si>
+  <si>
+    <t>PRATIBHA MAITI</t>
+  </si>
+  <si>
+    <t>MANAS RANJAN BHUNIA</t>
+  </si>
+  <si>
+    <t>AJIT MAITY</t>
+  </si>
+  <si>
+    <t>TAPAN BHUYA</t>
+  </si>
+  <si>
+    <t>RAJIB BANERJEE</t>
+  </si>
+  <si>
+    <t>ASHIS HUDAIT</t>
+  </si>
+  <si>
+    <t>SHYAMALI SARDAR</t>
+  </si>
+  <si>
+    <t>DOLOI SURJYA KANTA</t>
+  </si>
+  <si>
+    <t>UTTARA SINGHA (HAZRA)</t>
+  </si>
+  <si>
+    <t>SRIKANTA MAHATA</t>
+  </si>
+  <si>
+    <t>SUVENDU SAMANTA</t>
+  </si>
+  <si>
+    <t>SUJOY HAZRA</t>
+  </si>
+  <si>
+    <t>BIRBAHA HANSDA</t>
+  </si>
+  <si>
+    <t>RAJIB LOCHAN SAREN</t>
+  </si>
+  <si>
+    <t>SHANTIRAM MAHATO</t>
+  </si>
+  <si>
+    <t>SUSHANTA MAHATO</t>
+  </si>
+  <si>
+    <t>ARJUN MAHATO</t>
+  </si>
+  <si>
+    <t>SUJOY BANERJEE</t>
+  </si>
+  <si>
+    <t>SANDHYA RANI TUDU</t>
+  </si>
+  <si>
+    <t>SOUMEN BELTHARIA</t>
+  </si>
+  <si>
+    <t>MANIK CHANDRA BAURI</t>
+  </si>
+  <si>
+    <t>HAZARI BOURI</t>
+  </si>
+  <si>
+    <t>UTTAM BAURI</t>
+  </si>
+  <si>
+    <t>SWAPAN KUMAR MONDAL</t>
+  </si>
+  <si>
+    <t>TANUSHREE HANSDA</t>
+  </si>
+  <si>
+    <t>THAKURMANI SAREN</t>
+  </si>
+  <si>
+    <t>FALGUNI SINGHABABU</t>
+  </si>
+  <si>
+    <t>DR. ANUP MANDAL</t>
+  </si>
+  <si>
+    <t>GOUTAM MISHRA (SHYAM)</t>
+  </si>
+  <si>
+    <t>SUBRATA DUTTA (GOPI)</t>
+  </si>
+  <si>
+    <t>TANMAY GHOSH (BUMBA)</t>
+  </si>
+  <si>
+    <t>HARAKALI PROTIHER</t>
+  </si>
+  <si>
+    <t>SHYAMALI ROY BAGDI</t>
+  </si>
+  <si>
+    <t>KALLOL SAHA</t>
+  </si>
+  <si>
+    <t>GOUTAM DHARA</t>
+  </si>
+  <si>
     <t>KHOKAN DAS</t>
   </si>
   <si>
-    <t>DEBASIS OJHA (HAKU DA)</t>
-  </si>
-  <si>
-    <t>KRISHNA KANTA SAHA</t>
-  </si>
-  <si>
-    <t>DUDH KUMAR MONDAL</t>
-  </si>
-  <si>
-    <t>DHRUBA SAHA</t>
-  </si>
-  <si>
-    <t>FAYEZUL HAQUE (KAJAL SK)</t>
-  </si>
-  <si>
-    <t>RAJENDRA PRASAD SINGH(RAJU SINGH)</t>
-  </si>
-  <si>
-    <t>DR. MOSARRAF HOSSAIN</t>
-  </si>
-  <si>
-    <t>Bharatiya Janata Party</t>
-  </si>
-  <si>
-    <t>All India Trinamool Congress</t>
-  </si>
-  <si>
-    <t>Indian National Congress</t>
-  </si>
-  <si>
-    <t>Aam Janata Unnayan party</t>
-  </si>
-  <si>
-    <t>Communist Party of India (Marxist)</t>
-  </si>
-  <si>
-    <t>All India Secular Front</t>
-  </si>
-  <si>
-    <t>Won</t>
-  </si>
-  <si>
-    <t>Leading</t>
-  </si>
-  <si>
-    <t>ADHIKARY PARESH CHANDRA</t>
-  </si>
-  <si>
-    <t>DR. SABLU BARMAN</t>
-  </si>
-  <si>
-    <t>PARTHA PRATIM RAY</t>
-  </si>
-  <si>
-    <t>AVIJIT DE BHOWMIK</t>
-  </si>
-  <si>
-    <t>HARIHAR DAS</t>
-  </si>
-  <si>
-    <t>ASHUTOSH BARMA</t>
-  </si>
-  <si>
-    <t>UDAYAN GUHA</t>
-  </si>
-  <si>
-    <t>SAILENDRA NATH BARMA</t>
-  </si>
-  <si>
-    <t>SHIBSANKAR PAUL</t>
-  </si>
-  <si>
-    <t>RAJEEV TIRKEY</t>
-  </si>
-  <si>
-    <t>BIRENDRA BARA (ORAON)</t>
-  </si>
-  <si>
-    <t>SUMAN KANJILAL</t>
-  </si>
-  <si>
-    <t>SUBHASH CHANDRA ROY</t>
-  </si>
-  <si>
-    <t>JAYPRAKASH TOPPO</t>
-  </si>
-  <si>
-    <t>NIRMAL CHANDRA ROY</t>
-  </si>
-  <si>
-    <t>RAMMOHAN RAY</t>
-  </si>
-  <si>
-    <t>KRISHNA DAS</t>
-  </si>
-  <si>
-    <t>SWAPNA BARMAN</t>
-  </si>
-  <si>
-    <t>RANJAN SIL SHARMA</t>
-  </si>
-  <si>
-    <t>BULU CHIK BARAIK</t>
-  </si>
-  <si>
-    <t>SANJAY KUJUR</t>
-  </si>
-  <si>
-    <t>RUDEN SADA LEPCHA</t>
-  </si>
-  <si>
-    <t>BIJOY KUMAR RAI</t>
-  </si>
-  <si>
-    <t>AMAR LAMA</t>
-  </si>
-  <si>
-    <t>SHANKAR MALAKAR</t>
-  </si>
-  <si>
-    <t>GOUTAM DEB</t>
-  </si>
-  <si>
-    <t>REENA TOPNO EKKA</t>
-  </si>
-  <si>
-    <t>SANKAR ADHIKARI</t>
-  </si>
-  <si>
-    <t>CHITRAJIT ROY</t>
-  </si>
-  <si>
-    <t>SARAJIT BISWAS</t>
-  </si>
-  <si>
-    <t>MANOJ KUMAR JAIN</t>
-  </si>
-  <si>
-    <t>GOUTAM PAUL</t>
-  </si>
-  <si>
-    <t>SATYAJIT BARMAN</t>
-  </si>
-  <si>
-    <t>NITAI BAISHYA</t>
-  </si>
-  <si>
-    <t>KRISHNA KALYANI</t>
-  </si>
-  <si>
-    <t>SABITA BARMAN</t>
-  </si>
-  <si>
-    <t>REKHA ROY</t>
-  </si>
-  <si>
-    <t>SUBHENDU SARKAR</t>
-  </si>
-  <si>
-    <t>ARPITA GHOSH</t>
-  </si>
-  <si>
-    <t>CHINTAMANI BIHA</t>
-  </si>
-  <si>
-    <t>Goutam Das</t>
-  </si>
-  <si>
-    <t>DEBABRATA MAJUMDER</t>
-  </si>
-  <si>
-    <t>AMAL KISKU</t>
-  </si>
-  <si>
-    <t>PRASENJIT DAS</t>
-  </si>
-  <si>
-    <t>RATAN DAS</t>
-  </si>
-  <si>
-    <t>MAUSAM B NOOR</t>
-  </si>
-  <si>
-    <t>ABISHEK SINGHANIA</t>
-  </si>
-  <si>
-    <t>KABITA MANDAL</t>
-  </si>
-  <si>
-    <t>LIPIKA BARMAN GHOSH</t>
-  </si>
-  <si>
-    <t>ASIS KUNDU (PATA)</t>
-  </si>
-  <si>
-    <t>NIBARAN GHOSH</t>
-  </si>
-  <si>
-    <t>ABDUL HANNAN</t>
-  </si>
-  <si>
-    <t>CHANDANA SARKAR</t>
-  </si>
-  <si>
-    <t>SUNIL CHOWDHURI</t>
-  </si>
-  <si>
-    <t>MD NAJME ALAM</t>
-  </si>
-  <si>
-    <t>MAHABIR GHOSH</t>
-  </si>
-  <si>
-    <t>JAKIR HOSSAIN</t>
-  </si>
-  <si>
-    <t>NASIR SAIKH</t>
-  </si>
-  <si>
-    <t>TAPAS KUMAR CHAKRABORTY</t>
-  </si>
-  <si>
-    <t>TOUHIDUR RAHAMAN SUMAN</t>
-  </si>
-  <si>
-    <t>MAHAMUDAL HASAN</t>
-  </si>
-  <si>
-    <t>ABDUL SOUMIK HOSSAIN</t>
-  </si>
-  <si>
-    <t>SHAONI SINGHA ROY</t>
-  </si>
-  <si>
-    <t>PRONAB CHANDRA DAS</t>
-  </si>
-  <si>
-    <t>ASHIS MARJIT</t>
-  </si>
-  <si>
-    <t>PROTIMA RAJAK</t>
-  </si>
-  <si>
-    <t>APURBA SARKAR (DAVID)</t>
-  </si>
-  <si>
-    <t>ANAMIKA GHOSH</t>
-  </si>
-  <si>
-    <t>BAPAN GHOSH</t>
-  </si>
-  <si>
-    <t>RABIUL ALAM CHOWDHURY</t>
-  </si>
-  <si>
-    <t>ADHIR RANJAN CHOWDHURY</t>
-  </si>
-  <si>
-    <t>BIJOY SEKH</t>
-  </si>
-  <si>
-    <t>RANA MANDAL</t>
-  </si>
-  <si>
-    <t>IANUS ALI SARKAR</t>
-  </si>
-  <si>
-    <t>SOHAM CHAKRABORTY</t>
-  </si>
-  <si>
-    <t>DILIP KUMAR PODDAR</t>
-  </si>
-  <si>
-    <t>ANIMA DUTTA</t>
-  </si>
-  <si>
-    <t>KALLOL KHAN</t>
-  </si>
-  <si>
-    <t>SAIKAT SARKAR</t>
-  </si>
-  <si>
-    <t>SOMNATH DUTTA</t>
-  </si>
-  <si>
-    <t>PUNDARIKAKSHYA SAHA</t>
-  </si>
-  <si>
-    <t>UJJAL BISWAS</t>
-  </si>
-  <si>
-    <t>BRAJAKISHORE GOSWAMI</t>
-  </si>
-  <si>
-    <t>TAPAS KUMAR GHOSH</t>
-  </si>
-  <si>
-    <t>SAMIR KUMAR PODDAR</t>
-  </si>
-  <si>
-    <t>BARNALI DEY ROY</t>
-  </si>
-  <si>
-    <t>SOUGATA KUMAR BURMAN</t>
-  </si>
-  <si>
-    <t>SUBHANKAR SINGHA (JISHU)</t>
-  </si>
-  <si>
-    <t>DR. ATINDRA NATH MONDAL</t>
-  </si>
-  <si>
-    <t>DR. RAJIB BISWAS.</t>
-  </si>
-  <si>
-    <t>MADHUPARNA THAKUR</t>
-  </si>
-  <si>
-    <t>BISWAJIT DAS</t>
-  </si>
-  <si>
-    <t>RITUPARNA ADDHYA</t>
-  </si>
-  <si>
-    <t>NAROTTAM BISWAS</t>
-  </si>
-  <si>
-    <t>TARAK SAHA</t>
-  </si>
-  <si>
-    <t>SUKRITI KUMAR SARKAR</t>
-  </si>
-  <si>
-    <t>JYOTI PRIYA MALLICK</t>
-  </si>
-  <si>
-    <t>NARAYAN GOSWAMI</t>
-  </si>
-  <si>
-    <t>ARINDAM DEY</t>
-  </si>
-  <si>
-    <t>SUBODH ADHIKARY</t>
-  </si>
-  <si>
-    <t>SANAT DEY</t>
-  </si>
-  <si>
-    <t>AMIT GUPTA</t>
-  </si>
-  <si>
-    <t>SOMENATH SHYAM ICHINI</t>
-  </si>
-  <si>
-    <t>TRINANKUR BHATTACHARJEE</t>
-  </si>
-  <si>
-    <t>RAJ CHAKRABORTY (RAJU)</t>
-  </si>
-  <si>
-    <t>DEVADEEP PUROHIT</t>
-  </si>
-  <si>
-    <t>CHANDRIMA BHATTACHARYA</t>
-  </si>
-  <si>
-    <t>TIRTHANKAR GHOSH</t>
-  </si>
-  <si>
-    <t>ARUP CHOUDHURY (PULAK)</t>
-  </si>
-  <si>
-    <t>SAYANTIKA BANERJEE</t>
-  </si>
-  <si>
-    <t>BRATYABRATA BASU</t>
-  </si>
-  <si>
-    <t>PIYUSH KANODIA</t>
-  </si>
-  <si>
-    <t>SUJIT BOSE</t>
-  </si>
-  <si>
-    <t>ADITI MUNSHI</t>
-  </si>
-  <si>
-    <t>RATHIN GHOSH</t>
-  </si>
-  <si>
-    <t>SABYASACHI DUTTA</t>
-  </si>
-  <si>
-    <t>MD MOFIDUL HOQUE SAHAJI MINTU</t>
-  </si>
-  <si>
-    <t>PIYARUL ISLAM</t>
-  </si>
-  <si>
-    <t>RUDRENDRA PATRA</t>
-  </si>
-  <si>
-    <t>JHARNA SARDAR</t>
-  </si>
-  <si>
-    <t>DR. SOURYA BANERJEE</t>
-  </si>
-  <si>
-    <t>MD. MUSA KAREMULLA</t>
-  </si>
-  <si>
-    <t>ANANDA SARKAR</t>
-  </si>
-  <si>
-    <t>SUBRATA MONDAL</t>
-  </si>
-  <si>
-    <t>BIKASH SARDAR</t>
-  </si>
-  <si>
-    <t>MADHABI MAHALDER</t>
-  </si>
-  <si>
-    <t>ASIT KUMAR HALDAR</t>
-  </si>
-  <si>
-    <t>MANTURAM PAKHIRA</t>
-  </si>
-  <si>
-    <t>BANKIM CHANDRA HAZRA</t>
-  </si>
-  <si>
-    <t>ABANI NASKAR</t>
-  </si>
-  <si>
-    <t>PALASH RANA</t>
-  </si>
-  <si>
-    <t>MALLIKA PAIK W/O - ASHOK PAIK</t>
-  </si>
-  <si>
-    <t>ALOKE HALDER</t>
-  </si>
-  <si>
-    <t>TUMPA SARDAR</t>
-  </si>
-  <si>
-    <t>Prasanta Bayen</t>
-  </si>
-  <si>
-    <t>ARABUL ISLAM</t>
-  </si>
-  <si>
-    <t>BISWAJIT PAUL</t>
-  </si>
-  <si>
-    <t>UTTAM KUMAR BANIK</t>
-  </si>
-  <si>
-    <t>GOURSUNDAR GHOSH</t>
-  </si>
-  <si>
-    <t>DIPAK KUMAR HALDER</t>
-  </si>
-  <si>
-    <t>JAHANGIR KHAN</t>
-  </si>
-  <si>
-    <t>SOMASHREE BETAL</t>
-  </si>
-  <si>
-    <t>ABHIJIT SARDAR</t>
-  </si>
-  <si>
-    <t>ARUNDHUTI MAITRA(LOVELY)</t>
-  </si>
-  <si>
-    <t>SAOKAT MOLLA</t>
-  </si>
-  <si>
-    <t>BANERJEE SANDIP</t>
-  </si>
-  <si>
-    <t>DEBABRATA MAJUMDAR (MALAY)</t>
-  </si>
-  <si>
-    <t>FIRDOUSI BEGAM</t>
-  </si>
-  <si>
-    <t>AROOP BISWAS</t>
-  </si>
-  <si>
-    <t>SUBHASISH CHAKRABORTY</t>
-  </si>
-  <si>
-    <t>RATNA CHATTERJEE</t>
-  </si>
-  <si>
-    <t>TAMANATH BHOWMICK</t>
-  </si>
-  <si>
-    <t>DR TARUN KUMAR ADAK</t>
-  </si>
-  <si>
-    <t>BIR BAHADUR SINGH</t>
-  </si>
-  <si>
-    <t>RAKESH SINGH</t>
-  </si>
-  <si>
-    <t>MAMATA BANERJEE</t>
-  </si>
-  <si>
-    <t>DEBASISH KUMAR (DEBA)</t>
-  </si>
-  <si>
-    <t>SHATORUPA</t>
-  </si>
-  <si>
-    <t>SANTOSH KUMAR PATHAK</t>
-  </si>
-  <si>
-    <t>DR. PRIYANKA TIBREWAL</t>
-  </si>
-  <si>
-    <t>PARTHA CHAUDHURY</t>
-  </si>
-  <si>
-    <t>VIJAY UPADHYAY</t>
-  </si>
-  <si>
-    <t>SHASHI PANJA</t>
-  </si>
-  <si>
-    <t>SHRREYA PANDE</t>
-  </si>
-  <si>
-    <t>ATIN GHOSH</t>
-  </si>
-  <si>
-    <t>KAILASH KUMAR MISHRA</t>
-  </si>
-  <si>
-    <t>GAUTAM CHOWDHURY</t>
-  </si>
-  <si>
-    <t>BIPLAB KUMAR MANDAL</t>
-  </si>
-  <si>
-    <t>DR. RANA CHATTERJEE</t>
-  </si>
-  <si>
-    <t>SHYAMAL KUMAR HATI</t>
-  </si>
-  <si>
-    <t>BARNALI DHALI NASKAR</t>
-  </si>
-  <si>
-    <t>RANJAN PAUL</t>
-  </si>
-  <si>
-    <t>RUDRA PROSAD BANERJEE</t>
-  </si>
-  <si>
-    <t>BIMAL KUMAR DAS</t>
-  </si>
-  <si>
-    <t>SWAMI MANGALANANDA PURI</t>
-  </si>
-  <si>
-    <t>NADEBASI JANA</t>
-  </si>
-  <si>
-    <t>PRAMANSHU RANA</t>
-  </si>
-  <si>
-    <t>SUKANTA KUMAR PAUL</t>
-  </si>
-  <si>
-    <t>PROBHAKAR PANDIT</t>
-  </si>
-  <si>
-    <t>SUBIR CHATTERJEE (TINKAI)</t>
-  </si>
-  <si>
-    <t>GOBINDA HAZRA</t>
-  </si>
-  <si>
-    <t>SIRSANYA BANDOPADHYAY</t>
-  </si>
-  <si>
-    <t>TANMOY GHOSH</t>
-  </si>
-  <si>
-    <t>ARINDAM GUIN (BUBAI)</t>
-  </si>
-  <si>
-    <t>BECHARAM MANNA</t>
-  </si>
-  <si>
-    <t>Indranil Sen</t>
-  </si>
-  <si>
-    <t>DEBANGSHU BHATTACHARYA</t>
-  </si>
-  <si>
-    <t>RANJAN DHARA</t>
-  </si>
-  <si>
-    <t>SAMIR CHAKRABORTY</t>
-  </si>
-  <si>
-    <t>BIDESH RANJAN BOSE</t>
-  </si>
-  <si>
-    <t>DEBASISH MUKHERJEE</t>
-  </si>
-  <si>
-    <t>SNEHASIS CHAKRABORTY</t>
-  </si>
-  <si>
-    <t>KARABI MANNA</t>
-  </si>
-  <si>
-    <t>BARNALI DAS</t>
-  </si>
-  <si>
-    <t>RAMENDU SINHARAY</t>
-  </si>
-  <si>
-    <t>PARTHA HAZARI</t>
-  </si>
-  <si>
-    <t>BAG MITA</t>
-  </si>
-  <si>
-    <t>DR. NIRMAL MAJI</t>
-  </si>
-  <si>
-    <t>PALASH KUMAR ROY</t>
-  </si>
-  <si>
-    <t>DIPENDRA NARAYAN ROY</t>
-  </si>
-  <si>
-    <t>ASHIM KUMAR MAJI</t>
-  </si>
-  <si>
-    <t>SIRAJ KHAN</t>
-  </si>
-  <si>
-    <t>CHANDAN MONDAL</t>
-  </si>
-  <si>
-    <t>SUKUMAR DE</t>
-  </si>
-  <si>
-    <t>TILAK KUMAR CHAKRABORTY</t>
-  </si>
-  <si>
-    <t>TAPASI MONDAL</t>
-  </si>
-  <si>
-    <t>PABITRA KAR</t>
-  </si>
-  <si>
-    <t>UTTAM BARIK</t>
-  </si>
-  <si>
-    <t>PIJUS KANTI PANDA</t>
-  </si>
-  <si>
-    <t>DEBASIS BHUNYA</t>
-  </si>
-  <si>
-    <t>MANAB KUMAR PARUA</t>
-  </si>
-  <si>
-    <t>RABIN CHANDRA MANDAL</t>
-  </si>
-  <si>
-    <t>TARUN KUMAR JANA</t>
-  </si>
-  <si>
-    <t>AKHIL GIRI</t>
-  </si>
-  <si>
-    <t>TARUN KUMAR MAITY</t>
-  </si>
-  <si>
-    <t>MANIK MAITI</t>
-  </si>
-  <si>
-    <t>DULAL MURMU</t>
-  </si>
-  <si>
-    <t>AJIT MAHATA</t>
-  </si>
-  <si>
-    <t>MONGAL SAREN</t>
-  </si>
-  <si>
-    <t>RAMJIBAN MANDI</t>
-  </si>
-  <si>
-    <t>PRADIP SARKAR</t>
-  </si>
-  <si>
-    <t>PRATIBHA MAITI</t>
-  </si>
-  <si>
-    <t>MANAS RANJAN BHUNIA</t>
-  </si>
-  <si>
-    <t>AJIT MAITY</t>
-  </si>
-  <si>
-    <t>TAPAN BHUYA</t>
-  </si>
-  <si>
-    <t>RAJIB BANERJEE</t>
-  </si>
-  <si>
-    <t>ASHIS HUDAIT</t>
-  </si>
-  <si>
-    <t>SHYAMALI SARDAR</t>
-  </si>
-  <si>
-    <t>DOLOI SURJYA KANTA</t>
-  </si>
-  <si>
-    <t>UTTARA SINGHA (HAZRA)</t>
-  </si>
-  <si>
-    <t>SRIKANTA MAHATA</t>
-  </si>
-  <si>
-    <t>SUVENDU SAMANTA</t>
-  </si>
-  <si>
-    <t>SUJOY HAZRA</t>
-  </si>
-  <si>
-    <t>BIRBAHA HANSDA</t>
-  </si>
-  <si>
-    <t>RAJIB LOCHAN SAREN</t>
-  </si>
-  <si>
-    <t>SHANTIRAM MAHATO</t>
-  </si>
-  <si>
-    <t>SUSHANTA MAHATO</t>
-  </si>
-  <si>
-    <t>ARJUN MAHATO</t>
-  </si>
-  <si>
-    <t>SUJOY BANERJEE</t>
-  </si>
-  <si>
-    <t>SANDHYA RANI TUDU</t>
-  </si>
-  <si>
-    <t>SOUMEN BELTHARIA</t>
-  </si>
-  <si>
-    <t>MANIK CHANDRA BAURI</t>
-  </si>
-  <si>
-    <t>HAZARI BOURI</t>
-  </si>
-  <si>
-    <t>UTTAM BAURI</t>
-  </si>
-  <si>
-    <t>SWAPAN KUMAR MONDAL</t>
-  </si>
-  <si>
-    <t>TANUSHREE HANSDA</t>
-  </si>
-  <si>
-    <t>THAKURMANI SAREN</t>
-  </si>
-  <si>
-    <t>FALGUNI SINGHABABU</t>
-  </si>
-  <si>
-    <t>DR. ANUP MANDAL</t>
-  </si>
-  <si>
-    <t>GOUTAM MISHRA (SHYAM)</t>
-  </si>
-  <si>
-    <t>SUBRATA DUTTA (GOPI)</t>
-  </si>
-  <si>
-    <t>TANMAY GHOSH (BUMBA)</t>
-  </si>
-  <si>
-    <t>HARAKALI PROTIHER</t>
-  </si>
-  <si>
-    <t>SHYAMALI ROY BAGDI</t>
-  </si>
-  <si>
-    <t>KALLOL SAHA</t>
-  </si>
-  <si>
-    <t>GOUTAM DHARA</t>
-  </si>
-  <si>
     <t>MANDIRA DALUI</t>
   </si>
   <si>
@@ -2685,9 +2688,6 @@
   </si>
   <si>
     <t>UJJAL CHATTERJEE</t>
-  </si>
-  <si>
-    <t>BIDHAN CHANDRA MAJHI</t>
   </si>
   <si>
     <t>ABHIJIT SINHA (RANA)</t>
@@ -4274,7 +4274,7 @@
         <v>23</v>
       </c>
       <c r="C4">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
         <v>312</v>
@@ -4283,10 +4283,10 @@
         <v>601</v>
       </c>
       <c r="F4">
-        <v>135473</v>
+        <v>155327</v>
       </c>
       <c r="G4" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H4">
         <f>F4-K4</f>
@@ -4299,10 +4299,10 @@
         <v>602</v>
       </c>
       <c r="K4">
-        <v>73257</v>
+        <v>84943</v>
       </c>
       <c r="L4" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M4" t="s">
         <v>903</v>
@@ -4311,10 +4311,10 @@
         <v>605</v>
       </c>
       <c r="O4">
-        <v>4463</v>
+        <v>5293</v>
       </c>
       <c r="P4" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -4529,7 +4529,7 @@
         <v>22</v>
       </c>
       <c r="C9">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
         <v>317</v>
@@ -4538,10 +4538,10 @@
         <v>601</v>
       </c>
       <c r="F9">
-        <v>124086</v>
+        <v>126911</v>
       </c>
       <c r="G9" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H9">
         <f>F9-K9</f>
@@ -4554,10 +4554,10 @@
         <v>602</v>
       </c>
       <c r="K9">
-        <v>88019</v>
+        <v>92298</v>
       </c>
       <c r="L9" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M9" t="s">
         <v>908</v>
@@ -4566,10 +4566,10 @@
         <v>605</v>
       </c>
       <c r="O9">
-        <v>6230</v>
+        <v>6606</v>
       </c>
       <c r="P9" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -4631,7 +4631,7 @@
         <v>24</v>
       </c>
       <c r="C11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
         <v>319</v>
@@ -4640,10 +4640,10 @@
         <v>601</v>
       </c>
       <c r="F11">
-        <v>138982</v>
+        <v>143044</v>
       </c>
       <c r="G11" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H11">
         <f>F11-K11</f>
@@ -4656,10 +4656,10 @@
         <v>602</v>
       </c>
       <c r="K11">
-        <v>87630</v>
+        <v>90167</v>
       </c>
       <c r="L11" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M11" t="s">
         <v>910</v>
@@ -4668,10 +4668,10 @@
         <v>1193</v>
       </c>
       <c r="O11">
-        <v>3980</v>
+        <v>4111</v>
       </c>
       <c r="P11" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -4733,7 +4733,7 @@
         <v>22</v>
       </c>
       <c r="C13">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
         <v>321</v>
@@ -4742,7 +4742,7 @@
         <v>601</v>
       </c>
       <c r="F13">
-        <v>122808</v>
+        <v>131687</v>
       </c>
       <c r="G13" t="s">
         <v>608</v>
@@ -4758,7 +4758,7 @@
         <v>602</v>
       </c>
       <c r="K13">
-        <v>64288</v>
+        <v>67609</v>
       </c>
       <c r="L13" t="s">
         <v>900</v>
@@ -4770,7 +4770,7 @@
         <v>605</v>
       </c>
       <c r="O13">
-        <v>6480</v>
+        <v>6819</v>
       </c>
       <c r="P13" t="s">
         <v>900</v>
@@ -5138,10 +5138,10 @@
         <v>35</v>
       </c>
       <c r="B21">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C21">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D21" t="s">
         <v>329</v>
@@ -5150,7 +5150,7 @@
         <v>601</v>
       </c>
       <c r="F21">
-        <v>110214</v>
+        <v>112095</v>
       </c>
       <c r="G21" t="s">
         <v>607</v>
@@ -5166,7 +5166,7 @@
         <v>602</v>
       </c>
       <c r="K21">
-        <v>94502</v>
+        <v>96603</v>
       </c>
       <c r="L21" t="s">
         <v>899</v>
@@ -5178,7 +5178,7 @@
         <v>605</v>
       </c>
       <c r="O21">
-        <v>5758</v>
+        <v>5831</v>
       </c>
       <c r="P21" t="s">
         <v>899</v>
@@ -6005,10 +6005,10 @@
         <v>52</v>
       </c>
       <c r="B38">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C38">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D38" t="s">
         <v>346</v>
@@ -6017,7 +6017,7 @@
         <v>601</v>
       </c>
       <c r="F38">
-        <v>96477</v>
+        <v>97437</v>
       </c>
       <c r="G38" t="s">
         <v>607</v>
@@ -6033,7 +6033,7 @@
         <v>602</v>
       </c>
       <c r="K38">
-        <v>87840</v>
+        <v>88374</v>
       </c>
       <c r="L38" t="s">
         <v>899</v>
@@ -6045,7 +6045,7 @@
         <v>1193</v>
       </c>
       <c r="O38">
-        <v>6840</v>
+        <v>6861</v>
       </c>
       <c r="P38" t="s">
         <v>899</v>
@@ -8099,7 +8099,7 @@
         <v>23</v>
       </c>
       <c r="C79">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D79" t="s">
         <v>386</v>
@@ -8108,10 +8108,10 @@
         <v>601</v>
       </c>
       <c r="F79">
-        <v>111417</v>
+        <v>112138</v>
       </c>
       <c r="G79" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H79">
         <f>F79-K79</f>
@@ -8124,10 +8124,10 @@
         <v>602</v>
       </c>
       <c r="K79">
-        <v>82344</v>
+        <v>83885</v>
       </c>
       <c r="L79" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M79" t="s">
         <v>977</v>
@@ -8136,10 +8136,10 @@
         <v>605</v>
       </c>
       <c r="O79">
-        <v>24202</v>
+        <v>25629</v>
       </c>
       <c r="P79" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="80" spans="1:16">
@@ -8504,10 +8504,10 @@
         <v>101</v>
       </c>
       <c r="B87">
+        <v>17</v>
+      </c>
+      <c r="C87">
         <v>16</v>
-      </c>
-      <c r="C87">
-        <v>15</v>
       </c>
       <c r="D87" t="s">
         <v>394</v>
@@ -8516,7 +8516,7 @@
         <v>601</v>
       </c>
       <c r="F87">
-        <v>116881</v>
+        <v>117157</v>
       </c>
       <c r="G87" t="s">
         <v>608</v>
@@ -8532,7 +8532,7 @@
         <v>602</v>
       </c>
       <c r="K87">
-        <v>72335</v>
+        <v>72464</v>
       </c>
       <c r="L87" t="s">
         <v>900</v>
@@ -8544,7 +8544,7 @@
         <v>605</v>
       </c>
       <c r="O87">
-        <v>11461</v>
+        <v>11511</v>
       </c>
       <c r="P87" t="s">
         <v>900</v>
@@ -8558,7 +8558,7 @@
         <v>16</v>
       </c>
       <c r="C88">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D88" t="s">
         <v>395</v>
@@ -8567,7 +8567,7 @@
         <v>601</v>
       </c>
       <c r="F88">
-        <v>109260</v>
+        <v>126250</v>
       </c>
       <c r="G88" t="s">
         <v>608</v>
@@ -8583,7 +8583,7 @@
         <v>602</v>
       </c>
       <c r="K88">
-        <v>61709</v>
+        <v>70098</v>
       </c>
       <c r="L88" t="s">
         <v>900</v>
@@ -8595,7 +8595,7 @@
         <v>605</v>
       </c>
       <c r="O88">
-        <v>8279</v>
+        <v>9998</v>
       </c>
       <c r="P88" t="s">
         <v>900</v>
@@ -9119,7 +9119,7 @@
         <v>16</v>
       </c>
       <c r="C99">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D99" t="s">
         <v>406</v>
@@ -9128,7 +9128,7 @@
         <v>602</v>
       </c>
       <c r="F99">
-        <v>92089</v>
+        <v>94449</v>
       </c>
       <c r="G99" t="s">
         <v>608</v>
@@ -9144,7 +9144,7 @@
         <v>601</v>
       </c>
       <c r="K99">
-        <v>77125</v>
+        <v>78394</v>
       </c>
       <c r="L99" t="s">
         <v>900</v>
@@ -9156,7 +9156,7 @@
         <v>605</v>
       </c>
       <c r="O99">
-        <v>37539</v>
+        <v>38295</v>
       </c>
       <c r="P99" t="s">
         <v>900</v>
@@ -9303,7 +9303,7 @@
         <v>899</v>
       </c>
       <c r="M102" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="N102" t="s">
         <v>606</v>
@@ -9323,7 +9323,7 @@
         <v>20</v>
       </c>
       <c r="C103">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D103" t="s">
         <v>410</v>
@@ -9332,10 +9332,10 @@
         <v>602</v>
       </c>
       <c r="F103">
-        <v>76429</v>
+        <v>81670</v>
       </c>
       <c r="G103" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H103">
         <f>F103-K103</f>
@@ -9348,10 +9348,10 @@
         <v>601</v>
       </c>
       <c r="K103">
-        <v>72610</v>
+        <v>78675</v>
       </c>
       <c r="L103" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M103" t="s">
         <v>1000</v>
@@ -9360,10 +9360,10 @@
         <v>606</v>
       </c>
       <c r="O103">
-        <v>44613</v>
+        <v>46181</v>
       </c>
       <c r="P103" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="104" spans="1:16">
@@ -9527,7 +9527,7 @@
         <v>11</v>
       </c>
       <c r="C107">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D107" t="s">
         <v>414</v>
@@ -9536,10 +9536,10 @@
         <v>601</v>
       </c>
       <c r="F107">
-        <v>71753</v>
+        <v>94351</v>
       </c>
       <c r="G107" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H107">
         <f>F107-K107</f>
@@ -9552,10 +9552,10 @@
         <v>602</v>
       </c>
       <c r="K107">
-        <v>57481</v>
+        <v>73442</v>
       </c>
       <c r="L107" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M107" t="s">
         <v>1004</v>
@@ -9564,10 +9564,10 @@
         <v>1192</v>
       </c>
       <c r="O107">
-        <v>7070</v>
+        <v>9062</v>
       </c>
       <c r="P107" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="108" spans="1:16">
@@ -9578,7 +9578,7 @@
         <v>14</v>
       </c>
       <c r="C108">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D108" t="s">
         <v>415</v>
@@ -9587,10 +9587,10 @@
         <v>601</v>
       </c>
       <c r="F108">
-        <v>79332</v>
+        <v>94415</v>
       </c>
       <c r="G108" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H108">
         <f>F108-K108</f>
@@ -9603,10 +9603,10 @@
         <v>602</v>
       </c>
       <c r="K108">
-        <v>62496</v>
+        <v>76759</v>
       </c>
       <c r="L108" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M108" t="s">
         <v>1005</v>
@@ -9615,10 +9615,10 @@
         <v>605</v>
       </c>
       <c r="O108">
-        <v>15597</v>
+        <v>17696</v>
       </c>
       <c r="P108" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="109" spans="1:16">
@@ -9986,7 +9986,7 @@
         <v>17</v>
       </c>
       <c r="C116">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D116" t="s">
         <v>423</v>
@@ -9995,7 +9995,7 @@
         <v>602</v>
       </c>
       <c r="F116">
-        <v>90558</v>
+        <v>104324</v>
       </c>
       <c r="G116" t="s">
         <v>608</v>
@@ -10011,7 +10011,7 @@
         <v>601</v>
       </c>
       <c r="K116">
-        <v>77779</v>
+        <v>102250</v>
       </c>
       <c r="L116" t="s">
         <v>900</v>
@@ -10023,7 +10023,7 @@
         <v>605</v>
       </c>
       <c r="O116">
-        <v>26833</v>
+        <v>31654</v>
       </c>
       <c r="P116" t="s">
         <v>900</v>
@@ -10139,7 +10139,7 @@
         <v>17</v>
       </c>
       <c r="C119">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D119" t="s">
         <v>426</v>
@@ -10148,7 +10148,7 @@
         <v>601</v>
       </c>
       <c r="F119">
-        <v>82596</v>
+        <v>86049</v>
       </c>
       <c r="G119" t="s">
         <v>608</v>
@@ -10164,7 +10164,7 @@
         <v>602</v>
       </c>
       <c r="K119">
-        <v>77056</v>
+        <v>85076</v>
       </c>
       <c r="L119" t="s">
         <v>900</v>
@@ -10176,7 +10176,7 @@
         <v>606</v>
       </c>
       <c r="O119">
-        <v>23014</v>
+        <v>28805</v>
       </c>
       <c r="P119" t="s">
         <v>900</v>
@@ -10442,10 +10442,10 @@
         <v>139</v>
       </c>
       <c r="B125">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C125">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D125" t="s">
         <v>432</v>
@@ -10454,7 +10454,7 @@
         <v>602</v>
       </c>
       <c r="F125">
-        <v>112802</v>
+        <v>112965</v>
       </c>
       <c r="G125" t="s">
         <v>607</v>
@@ -10470,7 +10470,7 @@
         <v>601</v>
       </c>
       <c r="K125">
-        <v>102957</v>
+        <v>103421</v>
       </c>
       <c r="L125" t="s">
         <v>899</v>
@@ -10482,7 +10482,7 @@
         <v>605</v>
       </c>
       <c r="O125">
-        <v>23700</v>
+        <v>23710</v>
       </c>
       <c r="P125" t="s">
         <v>899</v>
@@ -10955,7 +10955,7 @@
         <v>23</v>
       </c>
       <c r="C135">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D135" t="s">
         <v>442</v>
@@ -10964,10 +10964,10 @@
         <v>602</v>
       </c>
       <c r="F135">
-        <v>93881</v>
+        <v>118991</v>
       </c>
       <c r="G135" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H135">
         <f>F135-K135</f>
@@ -10980,10 +10980,10 @@
         <v>601</v>
       </c>
       <c r="K135">
-        <v>86407</v>
+        <v>113034</v>
       </c>
       <c r="L135" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M135" t="s">
         <v>1032</v>
@@ -10992,10 +10992,10 @@
         <v>605</v>
       </c>
       <c r="O135">
-        <v>17156</v>
+        <v>19160</v>
       </c>
       <c r="P135" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="136" spans="1:16">
@@ -11003,10 +11003,10 @@
         <v>150</v>
       </c>
       <c r="B136">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C136">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D136" t="s">
         <v>443</v>
@@ -11015,10 +11015,10 @@
         <v>602</v>
       </c>
       <c r="F136">
-        <v>85157</v>
+        <v>93686</v>
       </c>
       <c r="G136" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H136">
         <f>F136-K136</f>
@@ -11031,10 +11031,10 @@
         <v>601</v>
       </c>
       <c r="K136">
-        <v>83956</v>
+        <v>91691</v>
       </c>
       <c r="L136" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M136" t="s">
         <v>1033</v>
@@ -11043,10 +11043,10 @@
         <v>606</v>
       </c>
       <c r="O136">
-        <v>19483</v>
+        <v>21943</v>
       </c>
       <c r="P136" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="137" spans="1:16">
@@ -11066,7 +11066,7 @@
         <v>602</v>
       </c>
       <c r="F137">
-        <v>108050</v>
+        <v>108194</v>
       </c>
       <c r="G137" t="s">
         <v>607</v>
@@ -11082,7 +11082,7 @@
         <v>601</v>
       </c>
       <c r="K137">
-        <v>81421</v>
+        <v>81844</v>
       </c>
       <c r="L137" t="s">
         <v>899</v>
@@ -11094,7 +11094,7 @@
         <v>605</v>
       </c>
       <c r="O137">
-        <v>18127</v>
+        <v>18151</v>
       </c>
       <c r="P137" t="s">
         <v>899</v>
@@ -11117,7 +11117,7 @@
         <v>602</v>
       </c>
       <c r="F138">
-        <v>109166</v>
+        <v>109625</v>
       </c>
       <c r="G138" t="s">
         <v>608</v>
@@ -11133,7 +11133,7 @@
         <v>601</v>
       </c>
       <c r="K138">
-        <v>83335</v>
+        <v>83820</v>
       </c>
       <c r="L138" t="s">
         <v>900</v>
@@ -11145,7 +11145,7 @@
         <v>605</v>
       </c>
       <c r="O138">
-        <v>17622</v>
+        <v>17713</v>
       </c>
       <c r="P138" t="s">
         <v>900</v>
@@ -11363,7 +11363,7 @@
         <v>19</v>
       </c>
       <c r="C143">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D143" t="s">
         <v>450</v>
@@ -11372,10 +11372,10 @@
         <v>602</v>
       </c>
       <c r="F143">
-        <v>100474</v>
+        <v>113834</v>
       </c>
       <c r="G143" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H143">
         <f>F143-K143</f>
@@ -11388,10 +11388,10 @@
         <v>601</v>
       </c>
       <c r="K143">
-        <v>45102</v>
+        <v>55331</v>
       </c>
       <c r="L143" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M143" t="s">
         <v>1040</v>
@@ -11400,10 +11400,10 @@
         <v>606</v>
       </c>
       <c r="O143">
-        <v>27261</v>
+        <v>28714</v>
       </c>
       <c r="P143" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="144" spans="1:16">
@@ -11414,7 +11414,7 @@
         <v>22</v>
       </c>
       <c r="C144">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D144" t="s">
         <v>451</v>
@@ -11423,7 +11423,7 @@
         <v>602</v>
       </c>
       <c r="F144">
-        <v>91094</v>
+        <v>104847</v>
       </c>
       <c r="G144" t="s">
         <v>608</v>
@@ -11439,7 +11439,7 @@
         <v>601</v>
       </c>
       <c r="K144">
-        <v>50391</v>
+        <v>68156</v>
       </c>
       <c r="L144" t="s">
         <v>900</v>
@@ -11451,7 +11451,7 @@
         <v>605</v>
       </c>
       <c r="O144">
-        <v>13644</v>
+        <v>15777</v>
       </c>
       <c r="P144" t="s">
         <v>900</v>
@@ -11516,7 +11516,7 @@
         <v>18</v>
       </c>
       <c r="C146">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D146" t="s">
         <v>453</v>
@@ -11525,10 +11525,10 @@
         <v>601</v>
       </c>
       <c r="F146">
-        <v>111016</v>
+        <v>111023</v>
       </c>
       <c r="G146" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H146">
         <f>F146-K146</f>
@@ -11541,10 +11541,10 @@
         <v>602</v>
       </c>
       <c r="K146">
-        <v>109975</v>
+        <v>110622</v>
       </c>
       <c r="L146" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M146" t="s">
         <v>1043</v>
@@ -11553,10 +11553,10 @@
         <v>605</v>
       </c>
       <c r="O146">
-        <v>11718</v>
+        <v>11736</v>
       </c>
       <c r="P146" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="147" spans="1:16">
@@ -11627,7 +11627,7 @@
         <v>601</v>
       </c>
       <c r="F148">
-        <v>128682</v>
+        <v>128970</v>
       </c>
       <c r="G148" t="s">
         <v>607</v>
@@ -11643,7 +11643,7 @@
         <v>602</v>
       </c>
       <c r="K148">
-        <v>92969</v>
+        <v>93188</v>
       </c>
       <c r="L148" t="s">
         <v>899</v>
@@ -11655,7 +11655,7 @@
         <v>1197</v>
       </c>
       <c r="O148">
-        <v>16751</v>
+        <v>16784</v>
       </c>
       <c r="P148" t="s">
         <v>899</v>
@@ -11771,7 +11771,7 @@
         <v>26</v>
       </c>
       <c r="C151">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D151" t="s">
         <v>458</v>
@@ -11780,10 +11780,10 @@
         <v>601</v>
       </c>
       <c r="F151">
-        <v>92412</v>
+        <v>106199</v>
       </c>
       <c r="G151" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H151">
         <f>F151-K151</f>
@@ -11796,10 +11796,10 @@
         <v>602</v>
       </c>
       <c r="K151">
-        <v>69307</v>
+        <v>78483</v>
       </c>
       <c r="L151" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M151" t="s">
         <v>1048</v>
@@ -11808,10 +11808,10 @@
         <v>605</v>
       </c>
       <c r="O151">
-        <v>35450</v>
+        <v>41148</v>
       </c>
       <c r="P151" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="152" spans="1:16">
@@ -11873,7 +11873,7 @@
         <v>17</v>
       </c>
       <c r="C153">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D153" t="s">
         <v>460</v>
@@ -11882,10 +11882,10 @@
         <v>601</v>
       </c>
       <c r="F153">
-        <v>88146</v>
+        <v>88407</v>
       </c>
       <c r="G153" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H153">
         <f>F153-K153</f>
@@ -11898,10 +11898,10 @@
         <v>602</v>
       </c>
       <c r="K153">
-        <v>82072</v>
+        <v>82394</v>
       </c>
       <c r="L153" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M153" t="s">
         <v>1050</v>
@@ -11910,10 +11910,10 @@
         <v>605</v>
       </c>
       <c r="O153">
-        <v>30237</v>
+        <v>30335</v>
       </c>
       <c r="P153" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="154" spans="1:16">
@@ -12230,7 +12230,7 @@
         <v>20</v>
       </c>
       <c r="C160">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D160" t="s">
         <v>467</v>
@@ -12239,10 +12239,10 @@
         <v>601</v>
       </c>
       <c r="F160">
-        <v>60954</v>
+        <v>73917</v>
       </c>
       <c r="G160" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H160">
         <f>F160-K160</f>
@@ -12255,10 +12255,10 @@
         <v>602</v>
       </c>
       <c r="K160">
-        <v>54728</v>
+        <v>58812</v>
       </c>
       <c r="L160" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M160" t="s">
         <v>1057</v>
@@ -12267,10 +12267,10 @@
         <v>605</v>
       </c>
       <c r="O160">
-        <v>2820</v>
+        <v>3556</v>
       </c>
       <c r="P160" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="161" spans="1:16">
@@ -12740,7 +12740,7 @@
         <v>15</v>
       </c>
       <c r="C170">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D170" t="s">
         <v>477</v>
@@ -12749,7 +12749,7 @@
         <v>601</v>
       </c>
       <c r="F170">
-        <v>44482</v>
+        <v>54588</v>
       </c>
       <c r="G170" t="s">
         <v>608</v>
@@ -12765,7 +12765,7 @@
         <v>602</v>
       </c>
       <c r="K170">
-        <v>34261</v>
+        <v>39734</v>
       </c>
       <c r="L170" t="s">
         <v>900</v>
@@ -12777,7 +12777,7 @@
         <v>605</v>
       </c>
       <c r="O170">
-        <v>9794</v>
+        <v>10831</v>
       </c>
       <c r="P170" t="s">
         <v>900</v>
@@ -13298,10 +13298,10 @@
         <v>195</v>
       </c>
       <c r="B181">
+        <v>20</v>
+      </c>
+      <c r="C181">
         <v>19</v>
-      </c>
-      <c r="C181">
-        <v>17</v>
       </c>
       <c r="D181" t="s">
         <v>488</v>
@@ -13310,7 +13310,7 @@
         <v>602</v>
       </c>
       <c r="F181">
-        <v>91442</v>
+        <v>104617</v>
       </c>
       <c r="G181" t="s">
         <v>608</v>
@@ -13326,7 +13326,7 @@
         <v>601</v>
       </c>
       <c r="K181">
-        <v>86335</v>
+        <v>93143</v>
       </c>
       <c r="L181" t="s">
         <v>900</v>
@@ -13338,7 +13338,7 @@
         <v>605</v>
       </c>
       <c r="O181">
-        <v>12317</v>
+        <v>13907</v>
       </c>
       <c r="P181" t="s">
         <v>900</v>
@@ -13349,10 +13349,10 @@
         <v>196</v>
       </c>
       <c r="B182">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C182">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D182" t="s">
         <v>489</v>
@@ -13361,7 +13361,7 @@
         <v>601</v>
       </c>
       <c r="F182">
-        <v>102983</v>
+        <v>104649</v>
       </c>
       <c r="G182" t="s">
         <v>607</v>
@@ -13377,7 +13377,7 @@
         <v>602</v>
       </c>
       <c r="K182">
-        <v>98995</v>
+        <v>100195</v>
       </c>
       <c r="L182" t="s">
         <v>899</v>
@@ -13389,7 +13389,7 @@
         <v>605</v>
       </c>
       <c r="O182">
-        <v>23111</v>
+        <v>23193</v>
       </c>
       <c r="P182" t="s">
         <v>899</v>
@@ -13400,10 +13400,10 @@
         <v>197</v>
       </c>
       <c r="B183">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C183">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D183" t="s">
         <v>490</v>
@@ -13412,10 +13412,10 @@
         <v>602</v>
       </c>
       <c r="F183">
-        <v>100333</v>
+        <v>105802</v>
       </c>
       <c r="G183" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H183">
         <f>F183-K183</f>
@@ -13428,10 +13428,10 @@
         <v>601</v>
       </c>
       <c r="K183">
-        <v>88401</v>
+        <v>93575</v>
       </c>
       <c r="L183" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M183" t="s">
         <v>1080</v>
@@ -13440,10 +13440,10 @@
         <v>605</v>
       </c>
       <c r="O183">
-        <v>7578</v>
+        <v>7849</v>
       </c>
       <c r="P183" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="184" spans="1:16">
@@ -13553,10 +13553,10 @@
         <v>200</v>
       </c>
       <c r="B186">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C186">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D186" t="s">
         <v>493</v>
@@ -13565,7 +13565,7 @@
         <v>601</v>
       </c>
       <c r="F186">
-        <v>80458</v>
+        <v>80612</v>
       </c>
       <c r="G186" t="s">
         <v>607</v>
@@ -13581,7 +13581,7 @@
         <v>602</v>
       </c>
       <c r="K186">
-        <v>70167</v>
+        <v>70197</v>
       </c>
       <c r="L186" t="s">
         <v>899</v>
@@ -13593,7 +13593,7 @@
         <v>605</v>
       </c>
       <c r="O186">
-        <v>49812</v>
+        <v>49820</v>
       </c>
       <c r="P186" t="s">
         <v>899</v>
@@ -13757,10 +13757,10 @@
         <v>204</v>
       </c>
       <c r="B190">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C190">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D190" t="s">
         <v>497</v>
@@ -13769,10 +13769,10 @@
         <v>601</v>
       </c>
       <c r="F190">
-        <v>78040</v>
+        <v>86273</v>
       </c>
       <c r="G190" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H190">
         <f>F190-K190</f>
@@ -13785,10 +13785,10 @@
         <v>602</v>
       </c>
       <c r="K190">
-        <v>67356</v>
+        <v>72832</v>
       </c>
       <c r="L190" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M190" t="s">
         <v>1087</v>
@@ -13797,10 +13797,10 @@
         <v>605</v>
       </c>
       <c r="O190">
-        <v>20695</v>
+        <v>22760</v>
       </c>
       <c r="P190" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="191" spans="1:16">
@@ -14063,10 +14063,10 @@
         <v>210</v>
       </c>
       <c r="B196">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C196">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D196" t="s">
         <v>503</v>
@@ -14075,10 +14075,10 @@
         <v>601</v>
       </c>
       <c r="F196">
-        <v>96953</v>
+        <v>102409</v>
       </c>
       <c r="G196" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H196">
         <f>F196-K196</f>
@@ -14091,10 +14091,10 @@
         <v>602</v>
       </c>
       <c r="K196">
-        <v>95765</v>
+        <v>101547</v>
       </c>
       <c r="L196" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M196" t="s">
         <v>1093</v>
@@ -14103,10 +14103,10 @@
         <v>605</v>
       </c>
       <c r="O196">
-        <v>17542</v>
+        <v>18138</v>
       </c>
       <c r="P196" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="197" spans="1:16">
@@ -14114,10 +14114,10 @@
         <v>211</v>
       </c>
       <c r="B197">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C197">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D197" t="s">
         <v>504</v>
@@ -14126,10 +14126,10 @@
         <v>601</v>
       </c>
       <c r="F197">
-        <v>102500</v>
+        <v>113332</v>
       </c>
       <c r="G197" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H197">
         <f>F197-K197</f>
@@ -14142,10 +14142,10 @@
         <v>602</v>
       </c>
       <c r="K197">
-        <v>99706</v>
+        <v>109844</v>
       </c>
       <c r="L197" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M197" t="s">
         <v>1094</v>
@@ -14154,10 +14154,10 @@
         <v>606</v>
       </c>
       <c r="O197">
-        <v>11562</v>
+        <v>12537</v>
       </c>
       <c r="P197" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="198" spans="1:16">
@@ -14573,10 +14573,10 @@
         <v>220</v>
       </c>
       <c r="B206">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C206">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D206" t="s">
         <v>513</v>
@@ -14585,10 +14585,10 @@
         <v>601</v>
       </c>
       <c r="F206">
-        <v>117861</v>
+        <v>137919</v>
       </c>
       <c r="G206" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H206">
         <f>F206-K206</f>
@@ -14601,10 +14601,10 @@
         <v>602</v>
       </c>
       <c r="K206">
-        <v>82808</v>
+        <v>105352</v>
       </c>
       <c r="L206" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M206" t="s">
         <v>1103</v>
@@ -14613,10 +14613,10 @@
         <v>606</v>
       </c>
       <c r="O206">
-        <v>7888</v>
+        <v>8702</v>
       </c>
       <c r="P206" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="207" spans="1:16">
@@ -14675,10 +14675,10 @@
         <v>222</v>
       </c>
       <c r="B208">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C208">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D208" t="s">
         <v>515</v>
@@ -14687,7 +14687,7 @@
         <v>601</v>
       </c>
       <c r="F208">
-        <v>131060</v>
+        <v>131476</v>
       </c>
       <c r="G208" t="s">
         <v>607</v>
@@ -14703,7 +14703,7 @@
         <v>602</v>
       </c>
       <c r="K208">
-        <v>100649</v>
+        <v>100873</v>
       </c>
       <c r="L208" t="s">
         <v>899</v>
@@ -14715,7 +14715,7 @@
         <v>605</v>
       </c>
       <c r="O208">
-        <v>9014</v>
+        <v>9020</v>
       </c>
       <c r="P208" t="s">
         <v>899</v>
@@ -14993,7 +14993,7 @@
         <v>601</v>
       </c>
       <c r="F214">
-        <v>118972</v>
+        <v>120227</v>
       </c>
       <c r="G214" t="s">
         <v>608</v>
@@ -15009,7 +15009,7 @@
         <v>602</v>
       </c>
       <c r="K214">
-        <v>103450</v>
+        <v>104537</v>
       </c>
       <c r="L214" t="s">
         <v>900</v>
@@ -15021,7 +15021,7 @@
         <v>605</v>
       </c>
       <c r="O214">
-        <v>4294</v>
+        <v>4375</v>
       </c>
       <c r="P214" t="s">
         <v>900</v>
@@ -15032,10 +15032,10 @@
         <v>229</v>
       </c>
       <c r="B215">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C215">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D215" t="s">
         <v>521</v>
@@ -15044,7 +15044,7 @@
         <v>601</v>
       </c>
       <c r="F215">
-        <v>129715</v>
+        <v>130586</v>
       </c>
       <c r="G215" t="s">
         <v>607</v>
@@ -15060,7 +15060,7 @@
         <v>602</v>
       </c>
       <c r="K215">
-        <v>109295</v>
+        <v>109708</v>
       </c>
       <c r="L215" t="s">
         <v>899</v>
@@ -15072,7 +15072,7 @@
         <v>1193</v>
       </c>
       <c r="O215">
-        <v>3655</v>
+        <v>3665</v>
       </c>
       <c r="P215" t="s">
         <v>899</v>
@@ -15086,7 +15086,7 @@
         <v>22</v>
       </c>
       <c r="C216">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D216" t="s">
         <v>522</v>
@@ -15095,10 +15095,10 @@
         <v>601</v>
       </c>
       <c r="F216">
-        <v>125212</v>
+        <v>129875</v>
       </c>
       <c r="G216" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H216">
         <f>F216-K216</f>
@@ -15111,10 +15111,10 @@
         <v>602</v>
       </c>
       <c r="K216">
-        <v>94041</v>
+        <v>97185</v>
       </c>
       <c r="L216" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M216" t="s">
         <v>1113</v>
@@ -15123,10 +15123,10 @@
         <v>605</v>
       </c>
       <c r="O216">
-        <v>5265</v>
+        <v>5365</v>
       </c>
       <c r="P216" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="217" spans="1:16">
@@ -15327,7 +15327,7 @@
         <v>1197</v>
       </c>
       <c r="O220">
-        <v>3581</v>
+        <v>3580</v>
       </c>
       <c r="P220" t="s">
         <v>899</v>
@@ -15545,7 +15545,7 @@
         <v>20</v>
       </c>
       <c r="C225">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D225" t="s">
         <v>530</v>
@@ -15554,10 +15554,10 @@
         <v>601</v>
       </c>
       <c r="F225">
-        <v>88512</v>
+        <v>89885</v>
       </c>
       <c r="G225" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H225">
         <f>F225-K225</f>
@@ -15570,10 +15570,10 @@
         <v>602</v>
       </c>
       <c r="K225">
-        <v>57413</v>
+        <v>59379</v>
       </c>
       <c r="L225" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M225" t="s">
         <v>1122</v>
@@ -15582,10 +15582,10 @@
         <v>605</v>
       </c>
       <c r="O225">
-        <v>5376</v>
+        <v>5451</v>
       </c>
       <c r="P225" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="226" spans="1:16">
@@ -17400,7 +17400,7 @@
         <v>0</v>
       </c>
       <c r="I261" t="s">
-        <v>593</v>
+        <v>865</v>
       </c>
       <c r="J261" t="s">
         <v>602</v>
@@ -17451,7 +17451,7 @@
         <v>0</v>
       </c>
       <c r="I262" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="J262" t="s">
         <v>602</v>
@@ -17502,7 +17502,7 @@
         <v>0</v>
       </c>
       <c r="I263" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="J263" t="s">
         <v>602</v>
@@ -17553,7 +17553,7 @@
         <v>0</v>
       </c>
       <c r="I264" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="J264" t="s">
         <v>602</v>
@@ -17604,7 +17604,7 @@
         <v>0</v>
       </c>
       <c r="I265" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="J265" t="s">
         <v>602</v>
@@ -17655,7 +17655,7 @@
         <v>0</v>
       </c>
       <c r="I266" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="J266" t="s">
         <v>602</v>
@@ -17687,7 +17687,7 @@
         <v>16</v>
       </c>
       <c r="C267">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D267" t="s">
         <v>572</v>
@@ -17696,7 +17696,7 @@
         <v>602</v>
       </c>
       <c r="F267">
-        <v>74796</v>
+        <v>107832</v>
       </c>
       <c r="G267" t="s">
         <v>608</v>
@@ -17706,13 +17706,13 @@
         <v>0</v>
       </c>
       <c r="I267" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="J267" t="s">
         <v>601</v>
       </c>
       <c r="K267">
-        <v>60328</v>
+        <v>98625</v>
       </c>
       <c r="L267" t="s">
         <v>900</v>
@@ -17724,7 +17724,7 @@
         <v>605</v>
       </c>
       <c r="O267">
-        <v>12361</v>
+        <v>18579</v>
       </c>
       <c r="P267" t="s">
         <v>900</v>
@@ -17757,7 +17757,7 @@
         <v>0</v>
       </c>
       <c r="I268" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="J268" t="s">
         <v>602</v>
@@ -17808,7 +17808,7 @@
         <v>0</v>
       </c>
       <c r="I269" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="J269" t="s">
         <v>602</v>
@@ -17859,7 +17859,7 @@
         <v>0</v>
       </c>
       <c r="I270" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="J270" t="s">
         <v>602</v>
@@ -17910,7 +17910,7 @@
         <v>0</v>
       </c>
       <c r="I271" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="J271" t="s">
         <v>602</v>
@@ -17961,7 +17961,7 @@
         <v>0</v>
       </c>
       <c r="I272" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="J272" t="s">
         <v>602</v>
@@ -18012,7 +18012,7 @@
         <v>0</v>
       </c>
       <c r="I273" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="J273" t="s">
         <v>602</v>
@@ -18063,7 +18063,7 @@
         <v>0</v>
       </c>
       <c r="I274" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="J274" t="s">
         <v>602</v>
@@ -18114,7 +18114,7 @@
         <v>0</v>
       </c>
       <c r="I275" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="J275" t="s">
         <v>602</v>
@@ -18165,7 +18165,7 @@
         <v>0</v>
       </c>
       <c r="I276" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="J276" t="s">
         <v>602</v>
@@ -18216,7 +18216,7 @@
         <v>0</v>
       </c>
       <c r="I277" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="J277" t="s">
         <v>602</v>
@@ -18267,7 +18267,7 @@
         <v>0</v>
       </c>
       <c r="I278" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="J278" t="s">
         <v>602</v>
@@ -18318,7 +18318,7 @@
         <v>0</v>
       </c>
       <c r="I279" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="J279" t="s">
         <v>602</v>
@@ -18369,7 +18369,7 @@
         <v>0</v>
       </c>
       <c r="I280" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="J280" t="s">
         <v>602</v>
@@ -18420,7 +18420,7 @@
         <v>0</v>
       </c>
       <c r="I281" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="J281" t="s">
         <v>602</v>
@@ -18471,7 +18471,7 @@
         <v>0</v>
       </c>
       <c r="I282" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="J282" t="s">
         <v>602</v>
@@ -18522,7 +18522,7 @@
         <v>0</v>
       </c>
       <c r="I283" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="J283" t="s">
         <v>602</v>
@@ -18573,7 +18573,7 @@
         <v>0</v>
       </c>
       <c r="I284" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="J284" t="s">
         <v>602</v>
@@ -18624,7 +18624,7 @@
         <v>0</v>
       </c>
       <c r="I285" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="J285" t="s">
         <v>602</v>
@@ -18653,10 +18653,10 @@
         <v>300</v>
       </c>
       <c r="B286">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C286">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D286" t="s">
         <v>591</v>
@@ -18665,26 +18665,26 @@
         <v>601</v>
       </c>
       <c r="F286">
-        <v>117754</v>
+        <v>124243</v>
       </c>
       <c r="G286" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H286">
         <f>F286-K286</f>
         <v>0</v>
       </c>
       <c r="I286" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="J286" t="s">
         <v>602</v>
       </c>
       <c r="K286">
-        <v>83964</v>
+        <v>95557</v>
       </c>
       <c r="L286" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M286" t="s">
         <v>1182</v>
@@ -18693,10 +18693,10 @@
         <v>605</v>
       </c>
       <c r="O286">
-        <v>7152</v>
+        <v>8064</v>
       </c>
       <c r="P286" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="287" spans="1:16">
@@ -18707,7 +18707,7 @@
         <v>23</v>
       </c>
       <c r="C287">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D287" t="s">
         <v>592</v>
@@ -18716,10 +18716,10 @@
         <v>602</v>
       </c>
       <c r="F287">
-        <v>109333</v>
+        <v>114915</v>
       </c>
       <c r="G287" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H287">
         <f>F287-K287</f>
@@ -18732,10 +18732,10 @@
         <v>601</v>
       </c>
       <c r="K287">
-        <v>95979</v>
+        <v>101727</v>
       </c>
       <c r="L287" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M287" t="s">
         <v>1183</v>
@@ -18744,10 +18744,10 @@
         <v>606</v>
       </c>
       <c r="O287">
-        <v>17526</v>
+        <v>18390</v>
       </c>
       <c r="P287" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="288" spans="1:16">
@@ -18758,35 +18758,35 @@
         <v>24</v>
       </c>
       <c r="C288">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D288" t="s">
         <v>593</v>
       </c>
       <c r="E288" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="F288">
-        <v>96177</v>
+        <v>119910</v>
       </c>
       <c r="G288" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H288">
         <f>F288-K288</f>
         <v>0</v>
       </c>
       <c r="I288" t="s">
-        <v>890</v>
+        <v>865</v>
       </c>
       <c r="J288" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="K288">
-        <v>89529</v>
+        <v>111788</v>
       </c>
       <c r="L288" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M288" t="s">
         <v>1184</v>
@@ -18795,10 +18795,10 @@
         <v>605</v>
       </c>
       <c r="O288">
-        <v>7278</v>
+        <v>10589</v>
       </c>
       <c r="P288" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="289" spans="1:16">
@@ -18806,10 +18806,10 @@
         <v>303</v>
       </c>
       <c r="B289">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C289">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D289" t="s">
         <v>594</v>
@@ -18818,7 +18818,7 @@
         <v>601</v>
       </c>
       <c r="F289">
-        <v>105830</v>
+        <v>106402</v>
       </c>
       <c r="G289" t="s">
         <v>607</v>
@@ -18834,7 +18834,7 @@
         <v>602</v>
       </c>
       <c r="K289">
-        <v>102647</v>
+        <v>102852</v>
       </c>
       <c r="L289" t="s">
         <v>899</v>
@@ -18846,7 +18846,7 @@
         <v>605</v>
       </c>
       <c r="O289">
-        <v>6152</v>
+        <v>6156</v>
       </c>
       <c r="P289" t="s">
         <v>899</v>
@@ -18962,7 +18962,7 @@
         <v>23</v>
       </c>
       <c r="C292">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D292" t="s">
         <v>597</v>
@@ -18971,10 +18971,10 @@
         <v>601</v>
       </c>
       <c r="F292">
-        <v>111249</v>
+        <v>111920</v>
       </c>
       <c r="G292" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H292">
         <f>F292-K292</f>
@@ -18987,10 +18987,10 @@
         <v>602</v>
       </c>
       <c r="K292">
-        <v>87335</v>
+        <v>87687</v>
       </c>
       <c r="L292" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M292" t="s">
         <v>1188</v>
@@ -18999,10 +18999,10 @@
         <v>605</v>
       </c>
       <c r="O292">
-        <v>22918</v>
+        <v>22994</v>
       </c>
       <c r="P292" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="293" spans="1:16">
@@ -19013,7 +19013,7 @@
         <v>21</v>
       </c>
       <c r="C293">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D293" t="s">
         <v>598</v>
@@ -19022,7 +19022,7 @@
         <v>602</v>
       </c>
       <c r="F293">
-        <v>81389</v>
+        <v>87827</v>
       </c>
       <c r="G293" t="s">
         <v>608</v>
@@ -19038,7 +19038,7 @@
         <v>601</v>
       </c>
       <c r="K293">
-        <v>43919</v>
+        <v>56684</v>
       </c>
       <c r="L293" t="s">
         <v>900</v>
@@ -19050,7 +19050,7 @@
         <v>605</v>
       </c>
       <c r="O293">
-        <v>19309</v>
+        <v>19796</v>
       </c>
       <c r="P293" t="s">
         <v>900</v>
@@ -19061,10 +19061,10 @@
         <v>308</v>
       </c>
       <c r="B294">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C294">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D294" t="s">
         <v>599</v>
@@ -19073,7 +19073,7 @@
         <v>602</v>
       </c>
       <c r="F294">
-        <v>65787</v>
+        <v>84854</v>
       </c>
       <c r="G294" t="s">
         <v>608</v>
@@ -19089,7 +19089,7 @@
         <v>601</v>
       </c>
       <c r="K294">
-        <v>59048</v>
+        <v>69715</v>
       </c>
       <c r="L294" t="s">
         <v>900</v>
@@ -19101,7 +19101,7 @@
         <v>603</v>
       </c>
       <c r="O294">
-        <v>29045</v>
+        <v>44425</v>
       </c>
       <c r="P294" t="s">
         <v>900</v>

</xml_diff>